<commit_message>
V2-M1 verified (CI 39083312122 and CodeQL green on fd0f556; clean clone 1977 tests, e2e 21/21); DEC-056: Shoaib named as the V2 qualified accountant (naming verifies nothing); V2 matrix v1.2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -3626,7 +3626,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>RECORDED 2026-10-17 (DEC-051..054, ADR-62..64)</t>
+          <t>RECORDED 2026-10-17 (DEC-051..054, ADR-62..64); qualified accountant named 2026-10-18: Shoaib (DEC-056)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>BUILT 2026-10-18 (acceptance package v2-m1-acceptance.md); rules unverified until the named accountant</t>
+          <t>ACCEPTED under the delegation 2026-10-18 (v2-m1-acceptance.md; CI 39083312122 on fd0f556); rules unverified until Shoaib verifies them (DEC-056)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -4053,7 +4053,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>fd0f556</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4061,7 +4065,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39083312122</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4086,7 +4094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4113,6 +4121,13 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>v1.2 (2026-10-18, DEC-056): V2-M1 evidence recorded (CI 39083312122 and CodeQL green on fd0f556; clean clone 1977 tests, e2e 21/21). Qualified accountant named: Shoaib; no row changes status from the naming alone.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V2-M2 verified (CI 39159238749 and CodeQL green on da32ffc; clean clone 2047 tests, e2e 21/21, OpenAPI drift 0); V2 matrix v1.3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -940,9 +940,9 @@
           <t>V2-M2</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -965,8 +965,16 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>packages/accounting/src/fixed-assets.ts; tests/golden/v2-m2-fixed-assets.json (hand figures; docs/architecture/v2-m2-golden-workings.xlsx recomputes all 37 independently: 0 differences); tests/api/fixed-assets.test.ts; tests/platform/fixed-assets.test.ts; tests/db/fixed-assets.test.ts</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>The register: classes, additions, depreciation, disposals, changes of estimate and the ledger reconciliation (V2-FA-01..08).</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -989,9 +997,9 @@
           <t>V2-M2</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1014,8 +1022,16 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>packages/accounting/src/depreciation-math.ts, fixed-assets.ts (DepreciationService); tests/api/fixed-assets.test.ts ('the golden scenario'); tests/platform/fixed-assets.test.ts ('FIXED_ASSET_DEPRECIATION and its reversal'); tests/rules/posting-rules.ts</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Runs post through the PostingService (FIXED_ASSET_DEPRECIATION): one journal, a pair of lines per class, one line per asset. A run must be later than every live run, one live run per date. Only the latest live run is reversed, by its own mirror. The source has its five test categories in the registry.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1585,9 +1601,9 @@
           <t>V2-M2</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1610,8 +1626,16 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>tests/golden/v2-m2-fixed-assets.json (hand figures; docs/architecture/v2-m2-golden-workings.xlsx recomputes all 37 independently: 0 differences); tests/api/fixed-assets.test.ts; tests/platform/fixed-assets.test.ts; tests/db/fixed-assets.test.ts</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Three kinds: POSTED (Dr cost / Cr a non-control offset), LINKED to the posting that already carries the cost (over-linking refused), TAKE_ON with accumulated depreciation. Reversal of a POSTED addition before any depreciation (VOID).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1634,9 +1658,9 @@
           <t>V2-M2</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1659,8 +1683,16 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr"/>
-      <c r="K23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>tests/golden/v2-m2-fixed-assets.json (hand figures; docs/architecture/v2-m2-golden-workings.xlsx recomputes all 37 independently: 0 differences); tests/api/fixed-assets.test.ts; tests/platform/fixed-assets.test.ts; tests/db/fixed-assets.test.ts</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Full disposals: catch-up to the disposal date, cost and accumulated depreciation removed, carrying amount and proceeds on the class disposal account; gain or loss = proceeds - carrying amount. Reversed by its mirror while no later run is live. Partial disposals are out of scope (DEC-058).</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1683,9 +1715,9 @@
           <t>V2-M2</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1708,8 +1740,16 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>packages/accounting/src/depreciation-math.ts; tests/unit/depreciation-math.test.ts; tests/golden/v2-m2-fixed-assets.json (hand figures; docs/architecture/v2-m2-golden-workings.xlsx recomputes all 37 independently: 0 differences); tests/api/fixed-assets.test.ts; tests/platform/fixed-assets.test.ts; tests/db/fixed-assets.test.ts</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Straight line and reducing balance, DAILY or MONTHLY convention; exact decimals; each charge = cumulative due (rounded half-up) - charged, so rounding never drifts.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1732,9 +1772,9 @@
           <t>V2-M2</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1757,8 +1797,16 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>tests/golden/v2-m2-fixed-assets.json (hand figures; docs/architecture/v2-m2-golden-workings.xlsx recomputes all 37 independently: 0 differences); tests/api/fixed-assets.test.ts; tests/platform/fixed-assets.test.ts; tests/db/fixed-assets.test.ts</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Life in months per class default or per asset; for a take-on, the remaining life; changed prospectively by a change of estimate (append-only bases).</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1781,9 +1829,9 @@
           <t>V2-M2</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1806,8 +1854,16 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>tests/golden/v2-m2-fixed-assets.json (hand figures; docs/architecture/v2-m2-golden-workings.xlsx recomputes all 37 independently: 0 differences); tests/api/fixed-assets.test.ts; tests/platform/fixed-assets.test.ts; tests/db/fixed-assets.test.ts</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Residual per asset (class default as a percentage of cost); straight line depreciates to it exactly; reducing balance never goes below it.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1830,9 +1886,9 @@
           <t>V2-M2</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1855,8 +1911,16 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>migration 20260120000000_v2_fixed_assets; tests/db/fixed-assets.test.ts ('classes'); tests/api/fixed-assets.test.ts ('classes name four accounts ...')</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>A class holds the four non-control accounts of the right type and subtype (database trigger) and the defaults for new assets; its code and accounts never move.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1879,9 +1943,9 @@
           <t>V2-M2</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1904,8 +1968,16 @@
           <t>Capital allowances computations (V4)</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>tests/unit/architecture.test.ts ('depreciation never reads the tax fields'); tests/api/fixed-assets.test.ts ('tax fields are stored apart')</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Tax category and tax cost stored on the asset for V4 (capital allowances); depreciation never reads them (architecture-tested); changing them changed no preview figure.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1928,9 +2000,9 @@
           <t>V2-M2</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1953,8 +2025,16 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>tests/api/fixed-assets.test.ts ('the register at 31.12.2026 ... reconciles', 'an unregistered posting ... reconciling item')</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Per cost and accumulated-depreciation account at a date: register against ledger, with every posting the register neither made nor linked listed as a reconciling item; golden reconciles to the cent, a manual posting shows as a 250.00 difference.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3712,7 +3792,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>ACCEPTED under the delegation 2026-10-18 (v2-m2-acceptance.md; CI 39159238749 on da32ffc)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -3727,7 +3807,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>to be specified before code</t>
+          <t>v2-plan.md section 4.4; v2-m2-acceptance.md</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -3739,7 +3819,7 @@
         <v>10</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -3994,7 +4074,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -4014,7 +4094,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>51</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5">
@@ -4044,7 +4124,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -4055,7 +4135,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>fd0f556</t>
+          <t>da32ffc</t>
         </is>
       </c>
     </row>
@@ -4067,7 +4147,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39083312122</t>
+          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39159238749</t>
         </is>
       </c>
     </row>
@@ -4094,7 +4174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4128,6 +4208,20 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>v1.3 (2026-10-18, V2-M2, DEC-057/058): fixed assets built. Missing -&gt; Implemented: V2-MOD-03, V2-MOD-04, V2-FA-01..08. Golden review of V2-M1 by Shoaib recorded (DEC-057); V2-TEST-01 stays Partially.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>v1.3a (2026-10-18): V2-M2 evidence recorded (CI 39159238749 and CodeQL 39159238888 green on da32ffc; clean clone 2047 tests, e2e 21/21, OpenAPI drift 0).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V2-M3a accepted: evidence recorded (CI 39178258465, CodeQL 39178258477 on f735149; clean clone 2091 tests, e2e 21/21, OpenAPI drift 0)
Matrix plan history v1.4a; milestone V2-M3 status updated (V2-M3a accepted, V2-M3b next).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -3920,7 +3920,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>SPLIT (DEC-059): V2-M3a adjustments BUILT 2026-10-18 (v2-m3a-acceptance.md); V2-M3b closing journal next</t>
+          <t>SPLIT (DEC-059): V2-M3a adjustments ACCEPTED under the delegation 2026-10-18 (v2-m3a-acceptance.md; CI 39178258465 on f735149); V2-M3b closing journal next</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -4218,7 +4218,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>f735149</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4226,7 +4230,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39178258465</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4236,7 +4244,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4306,6 +4314,13 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>v1.4a (2026-10-18): V2-M3a evidence recorded (CI 39178258465 and CodeQL 39178258477 green on f735149; clean clone 2091 tests, e2e 21/21, OpenAPI drift 0).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V2-M3b accepted: evidence recorded (CI 39181318428, CodeQL 39181318430 on 5ab27b8; clean clone 2117 tests, e2e 21/21, OpenAPI drift 0)
Matrix plan history v1.5a; milestone V2-M3 accepted (both halves).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -3924,7 +3924,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>SPLIT (DEC-059): V2-M3a adjustments ACCEPTED under the delegation 2026-10-18 (v2-m3a-acceptance.md; CI 39178258465 on f735149); V2-M3b closing journal BUILT 2026-10-19 (v2-m3b-acceptance.md)</t>
+          <t>ACCEPTED under the delegation (DEC-059 split): V2-M3a 2026-10-18 (v2-m3a-acceptance.md; CI 39178258465 on f735149); V2-M3b 2026-10-19 (v2-m3b-acceptance.md; CI 39181318428 on 5ab27b8)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -4222,7 +4222,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>5ab27b8</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4230,7 +4234,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39181318428</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4255,7 +4263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4324,6 +4332,13 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>v1.5a (2026-10-19): V2-M3b evidence recorded (CI 39181318428 and CodeQL 39181318430 green on 5ab27b8; clean clone 2117 tests, e2e 21/21, OpenAPI drift 0). Milestone V2-M3 accepted.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V2-M4 accepted: evidence recorded (CI 39251457210, CodeQL 39251456129 on 87c8956; clean clone 2146 tests, e2e 21/21, OpenAPI drift 0)
Matrix plan history v1.6a; milestone V2-M4 accepted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -3983,7 +3983,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>BUILT 2026-10-19 (v2-m4-acceptance.md)</t>
+          <t>ACCEPTED under the delegation 2026-10-19 (v2-m4-acceptance.md; CI 39251457210 on 87c8956)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -4238,7 +4238,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>87c8956</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4246,7 +4250,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39251457210</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4271,7 +4279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4354,6 +4362,13 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>v1.6a (2026-10-19): V2-M4 evidence recorded (CI 39251457210 and CodeQL 39251456129 green on 87c8956; clean clone 2146 tests, e2e 21/21, OpenAPI drift 0). A V1-M9a screen defect found by the first clean clone (a stale answer overwriting a newer one) was fixed in 87c8956.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V2-M5a accepted: evidence recorded (CI 39271179477, CodeQL 39271179462 on 1492ff6; clean clone 2163 tests, e2e 21/21, OpenAPI drift 0)
Matrix plan history v1.7a.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -4082,7 +4082,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>SPLIT (DEC-063): V2-M5a the accounts document BUILT 2026-10-19 (v2-m5a-acceptance.md); V2-M5b the size test and the cash flow statement next</t>
+          <t>SPLIT (DEC-063): V2-M5a the accounts document ACCEPTED under the delegation 2026-10-19 (v2-m5a-acceptance.md; CI 39271179477 on 1492ff6); V2-M5b the size test and the cash flow statement next</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -4294,7 +4294,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1492ff6</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4302,7 +4306,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39271179477</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4327,7 +4335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4424,6 +4432,13 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>v1.7a (2026-10-19): V2-M5a evidence recorded (CI 39271179477 and CodeQL 39271179462 green on 1492ff6; clean clone 2163 tests, e2e 21/21, OpenAPI drift 0).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Draft wording packs: evidence recorded (CI 39288936490, CodeQL 39288936669 on d08ecb3; clean clone 2175 tests, e2e 21/21)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -4294,7 +4294,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>d08ecb3</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4302,7 +4306,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39288936490</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4327,7 +4335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4438,6 +4446,13 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>v1.8a (2026-10-19): draft wording packs evidence recorded (CI 39288936490 and CodeQL 39288936669 green on d08ecb3; clean clone 2175 tests, e2e 21/21, OpenAPI drift 0).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V2-M5b accepted: evidence recorded (CI 39362598139, CodeQL 39362598131 on 2277775; clean clone 2204 tests, e2e 21/21, OpenAPI drift 0)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -4082,7 +4082,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>SPLIT (DEC-063, DEC-066): V2-M5a the accounts document ACCEPTED under the delegation 2026-10-19 (v2-m5a-acceptance.md; CI 39271179477 on 1492ff6); V2-M5b the size test built 2026-10-20 (v2-m5b-acceptance.md); V2-M5c the cash flow statement next</t>
+          <t>SPLIT (DEC-063, DEC-066): V2-M5a the accounts document ACCEPTED under the delegation 2026-10-19 (v2-m5a-acceptance.md; CI 39271179477 on 1492ff6); V2-M5b the size test ACCEPTED under the delegation 2026-10-20 (v2-m5b-acceptance.md; CI 39362598139 on 2277775); V2-M5c the cash flow statement next</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -4294,7 +4294,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2277775</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4302,7 +4306,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39362598139</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4327,7 +4335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4452,6 +4460,13 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>v1.9a (2026-10-20): V2-M5b evidence recorded (CI 39362598139 and CodeQL 39362598131 green on 2277775; clean clone 2204 tests, e2e 21/21, OpenAPI drift 0).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V2-M5c accepted: evidence recorded (CI 39396072282, CodeQL 39396072207 on 8fcee2c; clean clone 2225 tests, e2e 21/21, OpenAPI drift 0)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -4090,7 +4090,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>SPLIT (DEC-063, DEC-066): V2-M5a the accounts document ACCEPTED 2026-10-19 (v2-m5a-acceptance.md; CI 39271179477 on 1492ff6); V2-M5b the size test ACCEPTED 2026-10-20 (v2-m5b-acceptance.md; CI 39362598139 on 2277775); V2-M5c the cash flow statement built 2026-10-20 (v2-m5c-acceptance.md), all under the delegation</t>
+          <t>ACCEPTED under the delegation (DEC-063, DEC-066 split): V2-M5a the accounts document 2026-10-19 (v2-m5a-acceptance.md; CI 39271179477 on 1492ff6); V2-M5b the size test 2026-10-20 (v2-m5b-acceptance.md; CI 39362598139 on 2277775); V2-M5c the cash flow statement 2026-10-20 (v2-m5c-acceptance.md; CI 39396072282 on 8fcee2c)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -4302,7 +4302,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>8fcee2c</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4310,7 +4314,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39396072282</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4335,7 +4343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4474,6 +4482,13 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>v2.0a (2026-10-20): V2-M5c evidence recorded (CI 39396072282 and CodeQL 39396072207 green on 8fcee2c; clean clone 2225 tests, e2e 21/21, OpenAPI drift 0).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V2-M6a accepted: evidence recorded (CI 39575388052, CodeQL 39575387880 on 8646c7e; clean clone 2256 tests, e2e 21/21, OpenAPI drift 0)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -4213,7 +4213,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>SPLIT (DEC-068): V2-M6a review flags and the review checklist built 2026-10-21 (v2-m6a-acceptance.md); V2-M6b the 14-step year-end workflow and V2-M6c approval, locking and the filing-ready package next</t>
+          <t>SPLIT (DEC-068): V2-M6a review flags and the review checklist ACCEPTED under the delegation 2026-10-21 (v2-m6a-acceptance.md; CI 39575388052 on 8646c7e); V2-M6b the 14-step year-end workflow and V2-M6c approval, locking and the filing-ready package next</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -4382,7 +4382,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>8646c7e</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4390,7 +4394,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39575388052</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4415,7 +4423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4568,6 +4576,13 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>v2.1a (2026-10-21): V2-M6a evidence recorded (CI 39575388052 and CodeQL 39575387880 green on 8646c7e; clean clone 2256 tests, e2e 21/21, OpenAPI drift 0).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V2-M6b accepted: evidence recorded (CI 39595091384, CodeQL 39595091437 on 9868fbc; clean clone 2275 tests, e2e 21/21, OpenAPI drift 0)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -4321,7 +4321,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>SPLIT (DEC-068): V2-M6a review flags and the review checklist ACCEPTED 2026-10-21 (v2-m6a-acceptance.md; CI 39575388052 on 8646c7e); V2-M6b the 14-step year-end workflow built 2026-10-21 (v2-m6b-acceptance.md); V2-M6c approval, locking and the filing-ready package next</t>
+          <t>SPLIT (DEC-068): V2-M6a review flags and the review checklist ACCEPTED 2026-10-21 (v2-m6a-acceptance.md; CI 39575388052 on 8646c7e); V2-M6b the 14-step year-end workflow ACCEPTED 2026-10-21 (v2-m6b-acceptance.md; CI 39595091384 on 9868fbc); V2-M6c approval, locking and the filing-ready package next</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -4490,7 +4490,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>9868fbc</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4498,7 +4502,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39595091384</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4523,7 +4531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4690,6 +4698,13 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>v2.2a (2026-10-21): V2-M6b evidence recorded (CI 39595091384 and CodeQL 39595091437 green on 9868fbc; clean clone 2275 tests, e2e 21/21, OpenAPI drift 0).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V2-M6c: partner review, client approval, locking and the filing-ready package (DEC-070)
Specification recorded first (DEC-070, v2-plan 5j). The fingerprint of the
accounts document ties the records together: a second-person partner review
(lapses when the accounts change), the client's approval matching the approval
the accounts state (director, date, evidence), which locks the year's periods
through the period service and its framework, and a write-once filing-ready
package refused unless approved, unchanged and every rule verified (V2-ARC-04).
Database guards for each rule; steps 12-14 of the workflow done through their
own records (step 12 now waits for steps 1-11). Golden v2-m6c-approval (112
checks, 0 differences); V2-M6b golden revised with the revision recorded.
Matrix v2.3. Synthetic data only; not production approval.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -720,9 +720,9 @@
           <t>V2-M1</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -747,12 +747,12 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>tests/api/statutory.test.ts ('verification by a second person'); tests/db/reporting-framework.test.ts ('verification: once, by a person other than the author ...')</t>
+          <t>tests/api/statutory.test.ts ('verification by a second person'); tests/db/reporting-framework.test.ts ('verification: once, by a person other than the author ...'); tests/db/accounts-approval.test.ts ('the filing-ready package (V2-ARC-04) is refused under a version not verified by a second person ...'); tests/unit/accounts-approval.test.ts ('the package gate'); tests/api/accounts-approval.test.ts</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Built and tested: author cannot verify (service 403 and database CHECK), verified version and its content immutable (service 409 and database trigger), changes supersede, unverified previews carry verified=false and a PREVIEW ONLY notice. Remaining: the filing-ready refusal of unverified rules lands with V2-M6. No real rule is verified until the firm names its qualified accountant.</t>
+          <t>Built and tested. The author cannot verify (service 403 and database CHECK). A verified version and its content are immutable (service 409 and database trigger), and changes supersede. Unverified previews carry verified=false and a PREVIEW ONLY notice. Since V2-M6c (DEC-070), the filing-ready package is refused unless the standard version and every size threshold set used were verified by a second person (service), and the database refuses a package under a version never verified. This row is the mechanism only: no real standard content or threshold is verified yet. That is Shoaib's verification in the platform (DEC-052, DEC-056); "ok done" and document reviews verify nothing (DEC-065).</t>
         </is>
       </c>
     </row>
@@ -834,9 +834,9 @@
           <t>V2-M6</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -861,12 +861,12 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>tests/golden/v2-m6b-workflow.json (docs/architecture/v2-m6b-golden-workings.xlsx re-derives every control and state of five phases with an independent implementation of the rules: 79 checks, 0 differences); tests/api/year-end-workflow.test.ts; tests/unit/year-end-workflow.test.ts; tests/db/year-end-workflow.test.ts</t>
+          <t>tests/golden/v2-m6b-workflow.json (docs/architecture/v2-m6b-golden-workings.xlsx re-derives every control and state of five phases with an independent implementation of the rules: 79 checks, 0 differences); tests/api/year-end-workflow.test.ts; tests/unit/year-end-workflow.test.ts; tests/db/year-end-workflow.test.ts; tests/golden/v2-m6c-approval.json (docs/architecture/v2-m6c-golden-workings.xlsx re-derives every control, state and refusal of six phases with an independent implementation of the rules: 112 checks, 0 differences); tests/api/accounts-approval.test.ts; tests/unit/accounts-approval.test.ts; tests/db/accounts-approval.test.ts</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Built in V2-M6b (DEC-069): the 14-step workflow of a framework year with each step's control read from an existing control, its dependencies, its state (LATER, DONE, LAPSED, BLOCKED, TODO, ATTENTION), its sign-offs and the current step; steps 1 to 11 work end to end. Partially: steps 12 to 14 (partner review, client approval, the filing-ready package) arrive with V2-M6c.</t>
+          <t>Built in V2-M6b (DEC-069) and completed in V2-M6c (DEC-070): the 14-step workflow of a framework year. Each step's control is read from an existing control, with its dependencies, its state (DONE, LAPSED, BLOCKED, TODO, ATTENTION), its sign-offs or records, and the current step. Steps 1 to 11 are signed off by a preparer; steps 12 to 14 are done through the partner review, the client approval and the filing-ready package. Proven end to end on synthetic data.</t>
         </is>
       </c>
     </row>
@@ -1689,9 +1689,9 @@
           <t>V2-M6</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1714,8 +1714,16 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>tests/golden/v2-m6c-approval.json (docs/architecture/v2-m6c-golden-workings.xlsx re-derives every control, state and refusal of six phases with an independent implementation of the rules: 112 checks, 0 differences); tests/api/accounts-approval.test.ts; tests/unit/accounts-approval.test.ts; tests/db/accounts-approval.test.ts; tests/unit/architecture.test.ts ('approvals and packages have one writer ...')</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Built in V2-M6c (DEC-070). The partner review is recorded by a second person holding accounts:review, who is not the one who signed off the accounts (service 403 and database trigger), against the fingerprint (SHA-256) of the accounts document; it lapses when the accounts change. The client's approval is recorded with the approving director, the date and an evidence document, and must equal the approval the accounts state (Companies Act 2006 s.414). It needs a live partner review and the year's periods closed, and in the same transaction it locks the periods (through the period service) and the year's framework. After it, facts, flag responses, workflow sign-offs and reviews for the year are refused and its periods cannot be unlocked (service and database). Proven on synthetic data. Not built: withdrawing an approval and amended accounts (a later decision).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2821,9 +2829,9 @@
           <t>V2-M6</t>
         </is>
       </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2846,10 +2854,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>tests/golden/v2-m6c-approval.json (docs/architecture/v2-m6c-golden-workings.xlsx re-derives every control, state and refusal of six phases with an independent implementation of the rules: 112 checks, 0 differences); tests/api/accounts-approval.test.ts; tests/unit/accounts-approval.test.ts; tests/db/accounts-approval.test.ts</t>
+        </is>
+      </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Listed in the V2-M6b workflow as LATER (DEC-069); built with partner review, client approval and the filing-ready package in V2-M6c.</t>
+          <t>Built in V2-M6c (DEC-070): done through the partner review, not signed off in the workflow (step_own_record). Its control is the accounts document being complete and, once reviewed, unchanged since the review (READY, or ATTENTION when the accounts changed: LAPSED). Recorded by a second person with accounts:review, with time and an optional note. It is blocked until steps 1 to 11 are all done (DEC-070 amends DEC-069, which had it after step 11 alone). Proven on synthetic data.</t>
         </is>
       </c>
     </row>
@@ -2874,9 +2886,9 @@
           <t>V2-M6</t>
         </is>
       </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2899,10 +2911,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>tests/golden/v2-m6c-approval.json (docs/architecture/v2-m6c-golden-workings.xlsx re-derives every control, state and refusal of six phases with an independent implementation of the rules: 112 checks, 0 differences); tests/api/accounts-approval.test.ts; tests/unit/accounts-approval.test.ts; tests/db/accounts-approval.test.ts</t>
+        </is>
+      </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Listed in the V2-M6b workflow as LATER (DEC-069); built with partner review, client approval and the filing-ready package in V2-M6c.</t>
+          <t>Built in V2-M6c (DEC-070): done through the client approval. Its control is a live partner review, the year's periods closed and the approval facts set; once approved, the accounts unchanged since the approval. It records the director, the date, the evidence, who recorded it and when. Blocked until the partner review is done; it locks the year. Proven on synthetic data.</t>
         </is>
       </c>
     </row>
@@ -2927,9 +2943,9 @@
           <t>V2-M6</t>
         </is>
       </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2952,10 +2968,14 @@
           <t>iXBRL and Companies House filing (V3)</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>tests/golden/v2-m6c-approval.json (docs/architecture/v2-m6c-golden-workings.xlsx re-derives every control, state and refusal of six phases with an independent implementation of the rules: 112 checks, 0 differences); tests/api/accounts-approval.test.ts; tests/unit/accounts-approval.test.ts; tests/db/accounts-approval.test.ts</t>
+        </is>
+      </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Listed in the V2-M6b workflow as LATER (DEC-069); built with partner review, client approval and the filing-ready package in V2-M6c.</t>
+          <t>Built in V2-M6c (DEC-070): done through the filing-ready package, generated once per year by a preparer and stored write-once with its SHA-256. It holds the approved accounts document, the fingerprint, the framework and who verified it, the size test, the partner review and the client approval. It is refused unless the year is approved, the accounts are unchanged since then and every rule used was verified by a second person (V2-ARC-04). It is not a filing. Proven on synthetic data.</t>
         </is>
       </c>
     </row>
@@ -3919,12 +3939,12 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>tests/golden/v2-m1-micro-synthetic.json; tests/api/statutory.test.ts; tests/golden/v2-m2-fixed-assets.json; tests/golden/v2-m3a-adjustments.json; tests/golden/v2-m3b-close.json; tests/golden/v2-m4-directors.json; tests/golden/v2-m5a-document.json; tests/golden/v2-m5b-size.json; tests/golden/v2-m5c-cash-flow.json; tests/golden/v2-m6a-review.json; tests/golden/v2-m6b-workflow.json (each recomputed independently in its docs/architecture/v2-m*-golden-workings.xlsx)</t>
+          <t>tests/golden/v2-m1-micro-synthetic.json; tests/api/statutory.test.ts; tests/golden/v2-m2-fixed-assets.json; tests/golden/v2-m3a-adjustments.json; tests/golden/v2-m3b-close.json; tests/golden/v2-m4-directors.json; tests/golden/v2-m5a-document.json; tests/golden/v2-m5b-size.json; tests/golden/v2-m5c-cash-flow.json; tests/golden/v2-m6a-review.json; tests/golden/v2-m6b-workflow.json (each recomputed independently in its docs/architecture/v2-m*-golden-workings.xlsx); tests/golden/v2-m6c-approval.json</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>One micro-entity scenario with two layouts, written by hand first and matched to the cent. One hand figure (the broken-map net assets) was wrong on first run and recalculated by hand (recorded in the golden file). Remaining: scenarios for FRS 102 Section 1A and years with fixed assets and accruals (V2-M2..M5); review of the expected outputs by the named accountant before any real rule is verified. Since then each milestone added a hand-written golden scenario with an independent workbook (V2-M2 to V2-M6b, including the size test over four years and a medium-sized company's cash flow statement over two years); DEC-057 and DEC-061 record Shoaib's review of the V2-M1 to V2-M3b goldens. Still remaining: an FRS 102 Section 1A scenario and the named accountant's review of the V2-M4 to V2-M6b goldens.</t>
+          <t>One micro-entity scenario with two layouts, written by hand first and matched to the cent. One hand figure (the broken-map net assets) was wrong on first run and recalculated by hand (recorded in the golden file). Remaining: scenarios for FRS 102 Section 1A and years with fixed assets and accruals (V2-M2..M5); review of the expected outputs by the named accountant before any real rule is verified. Since then each milestone added a hand-written golden scenario with an independent workbook (V2-M2 to V2-M6c, including the size test over four years and a medium-sized company's cash flow statement over two years); DEC-057 and DEC-061 record Shoaib's review of the V2-M1 to V2-M3b goldens. Still remaining: an FRS 102 Section 1A scenario and the named accountant's review of the V2-M4 to V2-M6c goldens.</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4153,7 @@
         <v>9</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -4321,7 +4341,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>SPLIT (DEC-068): V2-M6a review flags and the review checklist ACCEPTED 2026-10-21 (v2-m6a-acceptance.md; CI 39575388052 on 8646c7e); V2-M6b the 14-step year-end workflow ACCEPTED 2026-10-21 (v2-m6b-acceptance.md; CI 39595091384 on 9868fbc); V2-M6c approval, locking and the filing-ready package next</t>
+          <t>SPLIT (DEC-068): V2-M6a review flags and the review checklist ACCEPTED 2026-10-21 (v2-m6a-acceptance.md; CI 39575388052 on 8646c7e); V2-M6b the 14-step year-end workflow ACCEPTED 2026-10-21 (v2-m6b-acceptance.md; CI 39595091384 on 9868fbc); V2-M6c partner review, client approval, locking and the filing-ready package BUILT 2026-10-21 (v2-m6c-acceptance.md, DEC-070), evidence pending</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -4336,7 +4356,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>v2-plan.md sections 5h.3 and 5i.4; v2-m6a-acceptance.md (V2-M6a); v2-m6b-acceptance.md (V2-M6b)</t>
+          <t>v2-plan.md sections 5h.3, 5i.4 and 5j.4; v2-m6a-acceptance.md (V2-M6a); v2-m6b-acceptance.md (V2-M6b); v2-m6c-acceptance.md (V2-M6c)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -4348,7 +4368,7 @@
         <v>26</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9">
@@ -4431,7 +4451,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3">
@@ -4441,7 +4461,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -4451,7 +4471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -4490,11 +4510,7 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>9868fbc</t>
-        </is>
-      </c>
+      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4502,11 +4518,7 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39595091384</t>
-        </is>
-      </c>
+      <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4531,7 +4543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4705,6 +4717,13 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>v2.3 (2026-10-21, V2-M6c, DEC-070): partner review, client approval, locking and the filing-ready package built. Missing -&gt; Implemented: V2-MOD-15, V2-YE-12 to V2-YE-14. Partially -&gt; Implemented: V2-MOD-01 (all 14 steps) and V2-ARC-04 (the filing-ready refusal of unverified rules; the mechanism only, no real rule verified). V2-TEST-01 gains the V2-M6c golden. The V2-M6b golden is revised for steps 12 to 14, with the revision recorded in the file. Proven on synthetic data.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V2-M6c accepted: evidence recorded (CI 39608223030, CodeQL 39608218001 on 120a949; clean clone 2302 tests, e2e 21/21, OpenAPI drift 0)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>SPLIT (DEC-068): V2-M6a review flags and the review checklist ACCEPTED 2026-10-21 (v2-m6a-acceptance.md; CI 39575388052 on 8646c7e); V2-M6b the 14-step year-end workflow ACCEPTED 2026-10-21 (v2-m6b-acceptance.md; CI 39595091384 on 9868fbc); V2-M6c partner review, client approval, locking and the filing-ready package BUILT 2026-10-21 (v2-m6c-acceptance.md, DEC-070), evidence pending</t>
+          <t>SPLIT (DEC-068): V2-M6a review flags and the review checklist ACCEPTED 2026-10-21 (v2-m6a-acceptance.md; CI 39575388052 on 8646c7e); V2-M6b the 14-step year-end workflow ACCEPTED 2026-10-21 (v2-m6b-acceptance.md; CI 39595091384 on 9868fbc); V2-M6c partner review, client approval, locking and the filing-ready package ACCEPTED 2026-10-21 (v2-m6c-acceptance.md, DEC-070; CI 39608223030 on 120a949)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -4510,7 +4510,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>120a949</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4518,7 +4522,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39608223030</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4543,7 +4551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4724,6 +4732,13 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>v2.3a (2026-10-21): V2-M6c evidence recorded (CI 39608223030 and CodeQL 39608218001 green on 120a949; clean clone 2302 tests, e2e 21/21, OpenAPI drift 0; the first push 0731c7e failed typecheck and was fixed in 120a949).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V2-M7 specification: split into three slices; V2-M7a the year-end workspace screens (DEC-071, v2-plan 5k)
Recorded before code. Screens show what the API returns and compute nothing;
each slice proven in a real browser (DEC-050).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -4384,7 +4384,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>SPLIT (DEC-071): V2-M7a the year-end workspace in progress (specified in v2-plan 5k); V2-M7b the registers and V2-M7c the reporting framework to be specified before their code</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -4399,7 +4399,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>to be specified before code</t>
+          <t>v2-plan.md section 5k (V2-M7a); DEC-050 real-browser proof per slice</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -4510,11 +4510,7 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>120a949</t>
-        </is>
-      </c>
+      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4522,11 +4518,7 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39608223030</t>
-        </is>
-      </c>
+      <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">

</xml_diff>

<commit_message>
V2-M7a: the year-end workspace screens (DEC-071, v2-plan 5k)
Year end (the 14-step workflow, sign-off and reopen), Review (the checklist,
explain/sign off/reopen, settings), Accounts (the accounts document, facts,
size test) and Approval (partner review, client approval with director and
evidence, the filing-ready package) behind accounts.production. The screens
show what the API returns and compute nothing. Proven in a real browser
(DEC-050): the main path to the package, a refusal shown in the API's words,
a reviewer with no action button, the feature off. Matrix v2.4 (V2-DOD-01
stays Missing until V2-M7b and V2-M7c).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -3994,8 +3994,16 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J62" s="2" t="inlineStr"/>
-      <c r="K62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>tests/e2e/year-end.test.ts (V2-M7a: the year-end workspace, five real-browser tests); docs/architecture/v2-m7a-acceptance.md (each screen with its API routes)</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>Split into three slices (DEC-071). V2-M7a, the year-end workspace, is built: the workflow, the review checklist and settings, the accounts document with its facts and size test, and the approval and package. It is behind accounts.production and proven in a real browser (DEC-050): the main path from step 11 to the package, a refusal shown in the API's words, a reviewer with no action button, and the feature off. Still missing: V2-M7b, the registers (fixed assets, year-end adjustments, the closing journal, director loans and related parties), and V2-M7c, the reporting framework (standards, verification, thresholds, the framework of each year, the statutory preview and cash flow). Those modules work through the API only, so the row stays Missing until all three slices are accepted.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K62"/>
@@ -4384,7 +4392,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>SPLIT (DEC-071): V2-M7a the year-end workspace in progress (specified in v2-plan 5k); V2-M7b the registers and V2-M7c the reporting framework to be specified before their code</t>
+          <t>SPLIT (DEC-071): V2-M7a the year-end workspace BUILT 2026-10-21 (v2-m7a-acceptance.md), evidence pending; V2-M7b the registers and V2-M7c the reporting framework to be specified before their code</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -4399,7 +4407,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>v2-plan.md section 5k (V2-M7a); DEC-050 real-browser proof per slice</t>
+          <t>v2-plan.md section 5k (V2-M7a); v2-m7a-acceptance.md; DEC-050 real-browser proof per slice</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -4543,7 +4551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4731,6 +4739,13 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>v2.4 (2026-10-21, V2-M7a, DEC-071): the year-end workspace screens built (workflow, review, accounts, approval and package) and proven in a real browser. V2-DOD-01 stays Missing until V2-M7b and V2-M7c; its note records the slice. No status change.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V2-M7a accepted: evidence recorded (CI 39660002000, CodeQL 39660002001 on 23b366f; clean clone 2302 tests, e2e 26/26, OpenAPI drift 0)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -4392,7 +4392,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>SPLIT (DEC-071): V2-M7a the year-end workspace BUILT 2026-10-21 (v2-m7a-acceptance.md), evidence pending; V2-M7b the registers and V2-M7c the reporting framework to be specified before their code</t>
+          <t>SPLIT (DEC-071): V2-M7a the year-end workspace ACCEPTED 2026-10-21 (v2-m7a-acceptance.md; CI 39660002000 on 23b366f); V2-M7b the registers and V2-M7c the reporting framework to be specified before their code</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -4518,7 +4518,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>23b366f</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4526,7 +4530,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39660002000</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4551,7 +4559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4746,6 +4754,13 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>v2.4a (2026-10-21): V2-M7a evidence recorded (CI 39660002000 and CodeQL 39660002001 green on 23b366f; clean clone 2302 tests, e2e 26/26, OpenAPI drift 0).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
DEC-072: engineering's data check of V2 (a review, not verification)
Goldens re-run (905 checks, 0 differences), 44 hand-written journals
balanced, V2-M1 statements recomputed in both layouts, 610 matrix evidence
paths present, draft size thresholds checked against reachable sources, every
reference in the wording packs assessed. One finding (NOTE.CREDLONG), five to
check, one not confirmed, one limitation. Nothing in the platform changed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -4518,11 +4518,7 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>23b366f</t>
-        </is>
-      </c>
+      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4530,11 +4526,7 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39660002000</t>
-        </is>
-      </c>
+      <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4559,7 +4551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4761,6 +4753,13 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>v2.4b (2026-10-21, DEC-072): engineering's data check (a review, not verification). Goldens 905 checks with 0 differences; 44 journals balanced; V2-M1 statements recomputed; 610 evidence paths present; thresholds confirmed against secondary sources; one wording finding (NOTE.CREDLONG). No status change.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V2-M7b specification: the register screens (DEC-074, v2-plan 5k.3)
Recorded before code.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -4392,7 +4392,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>SPLIT (DEC-071): V2-M7a the year-end workspace ACCEPTED 2026-10-21 (v2-m7a-acceptance.md; CI 39660002000 on 23b366f); V2-M7b the registers and V2-M7c the reporting framework to be specified before their code</t>
+          <t>SPLIT (DEC-071): V2-M7a the year-end workspace ACCEPTED 2026-10-21 (v2-m7a-acceptance.md; CI 39660002000 on 23b366f); V2-M7b the registers in progress (specified in v2-plan 5k.3, DEC-074); V2-M7c the reporting framework to be specified before its code</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>v2-plan.md section 5k (V2-M7a); v2-m7a-acceptance.md; DEC-050 real-browser proof per slice</t>
+          <t>v2-plan.md section 5k (V2-M7a); v2-m7a-acceptance.md; DEC-050 real-browser proof per slice; v2-plan.md section 5k.3 (V2-M7b)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
V2-M7b: the register screens (DEC-074, v2-plan 5k.3)
Fixed assets (register with reconciliation, classes, assets, each asset's
estimate, tax fields, disposal and reversals), depreciation runs, year-end
adjustments and release runs, provisions and movements, the closing journal,
director loan accounts (statement, report, thresholds) and related parties,
behind accounts.production. The screens show what the API returns and compute
nothing. Proven in a real browser (DEC-050): each register's main action, a
refusal shown in the API's words, a reviewer with no action button; the close
asserted against the hand figure (-800.00). Matrix v2.5 (V2-DOD-01 stays
Missing until V2-M7c).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -3996,12 +3996,12 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>tests/e2e/year-end.test.ts (V2-M7a: the year-end workspace, five real-browser tests); docs/architecture/v2-m7a-acceptance.md (each screen with its API routes)</t>
+          <t>tests/e2e/year-end.test.ts (V2-M7a: the year-end workspace, five real-browser tests); docs/architecture/v2-m7a-acceptance.md (each screen with its API routes); tests/e2e/registers.test.ts (V2-M7b: the registers, six real-browser tests); docs/architecture/v2-m7b-acceptance.md</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>Split into three slices (DEC-071). V2-M7a, the year-end workspace, is built: the workflow, the review checklist and settings, the accounts document with its facts and size test, and the approval and package. It is behind accounts.production and proven in a real browser (DEC-050): the main path from step 11 to the package, a refusal shown in the API's words, a reviewer with no action button, and the feature off. Still missing: V2-M7b, the registers (fixed assets, year-end adjustments, the closing journal, director loans and related parties), and V2-M7c, the reporting framework (standards, verification, thresholds, the framework of each year, the statutory preview and cash flow). Those modules work through the API only, so the row stays Missing until all three slices are accepted.</t>
+          <t>Split into three slices (DEC-071). V2-M7a, the year-end workspace, is built: the workflow, the review checklist and settings, the accounts document with its facts and size test, and the approval and package. It is behind accounts.production and proven in a real browser (DEC-050): the main path from step 11 to the package, a refusal shown in the API's words, a reviewer with no action button, and the feature off. V2-M7b, the registers, is built: fixed assets and each asset, depreciation, year-end adjustments and release runs, provisions, the closing journal, director loan accounts and related parties. Proven in a real browser: each register's main action, a refusal shown in the API's words, and a reviewer with no action button. Still missing: V2-M7c, the reporting framework (standards, verification, thresholds, the framework of each year, the statutory preview and cash flow). Those modules work through the API only, so the row stays Missing until V2-M7c is accepted.</t>
         </is>
       </c>
     </row>
@@ -4392,7 +4392,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>SPLIT (DEC-071): V2-M7a the year-end workspace ACCEPTED 2026-10-21 (v2-m7a-acceptance.md; CI 39660002000 on 23b366f); V2-M7b the registers in progress (specified in v2-plan 5k.3, DEC-074); V2-M7c the reporting framework to be specified before its code</t>
+          <t>SPLIT (DEC-071): V2-M7a the year-end workspace ACCEPTED 2026-10-21 (v2-m7a-acceptance.md; CI 39660002000 on 23b366f); V2-M7b the registers BUILT 2026-10-22 (v2-m7b-acceptance.md, DEC-074), evidence pending; V2-M7c the reporting framework to be specified before its code</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>v2-plan.md section 5k (V2-M7a); v2-m7a-acceptance.md; DEC-050 real-browser proof per slice; v2-plan.md section 5k.3 (V2-M7b)</t>
+          <t>v2-plan.md section 5k (V2-M7a); v2-m7a-acceptance.md; DEC-050 real-browser proof per slice; v2-plan.md section 5k.3 (V2-M7b); v2-m7b-acceptance.md</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -4551,7 +4551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4760,6 +4760,13 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>v2.5 (2026-10-22, V2-M7b, DEC-074): the register screens built (fixed assets, depreciation, adjustments, provisions, closing journal, directors, related parties) and proven in a real browser. V2-DOD-01 stays Missing until V2-M7c; its note records the slice. No status change.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V2-M7b accepted: evidence recorded (CI 39776060443, CodeQL 39776060387 on 2d53914; clean clone 2302 tests, e2e 32/32, OpenAPI drift 0)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-compliance-matrix.xlsx
+++ b/docs/architecture/v2-compliance-matrix.xlsx
@@ -4392,7 +4392,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>SPLIT (DEC-071): V2-M7a the year-end workspace ACCEPTED 2026-10-21 (v2-m7a-acceptance.md; CI 39660002000 on 23b366f); V2-M7b the registers BUILT 2026-10-22 (v2-m7b-acceptance.md, DEC-074), evidence pending; V2-M7c the reporting framework to be specified before its code</t>
+          <t>SPLIT (DEC-071): V2-M7a the year-end workspace ACCEPTED 2026-10-21 (v2-m7a-acceptance.md; CI 39660002000 on 23b366f); V2-M7b the registers ACCEPTED 2026-10-22 (v2-m7b-acceptance.md, DEC-074; CI 39776060443 on 2d53914); V2-M7c the reporting framework to be specified before its code</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -4518,7 +4518,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2d53914</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4526,7 +4530,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/39776060443</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4551,7 +4559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4767,6 +4775,13 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>v2.5a (2026-10-22): V2-M7b evidence recorded (CI 39776060443 and CodeQL 39776060387 green on 2d53914; clean clone 2302 tests, e2e 32/32, OpenAPI drift 0).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>